<commit_message>
fix: refine q3 v2 policy labels
</commit_message>
<xml_diff>
--- a/第三问_文化考察均衡优化材料包/10_Q3_V2_鲁棒三团队文化考察调度/reports/新疆旅游第三问Q3_V2鲁棒三团队文化考察结果.xlsx
+++ b/第三问_文化考察均衡优化材料包/10_Q3_V2_鲁棒三团队文化考察调度/reports/新疆旅游第三问Q3_V2鲁棒三团队文化考察结果.xlsx
@@ -2324,7 +2324,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>charter_car</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>taxi_transfer</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>taxi_transfer</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>charter_car</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>rental_car</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>charter_car</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>taxi_transfer</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>rental_car</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>charter_car</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>charter_car</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -3122,7 +3122,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>mixed_transfer</t>
+          <t>rental_car</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>楼兰古城 -&gt; 尼雅遗址；mixed_transfer</t>
+          <t>楼兰古城 -&gt; 尼雅遗址；charter_car</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3928,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>楼兰古城 -&gt; 尼雅遗址；mixed_transfer</t>
+          <t>楼兰古城 -&gt; 尼雅遗址；charter_car</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4556,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4788,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -5044,7 +5044,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>吐峪沟麻扎村 -&gt; 苏公塔；mixed_transfer</t>
+          <t>吐峪沟麻扎村 -&gt; 苏公塔；taxi_transfer</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>苏公塔 -&gt; 交河故城；mixed_transfer</t>
+          <t>苏公塔 -&gt; 交河故城；taxi_transfer</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>交河故城 -&gt; 罗布人村寨；mixed_transfer</t>
+          <t>交河故城 -&gt; 罗布人村寨；charter_car</t>
         </is>
       </c>
     </row>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>交河故城 -&gt; 罗布人村寨；mixed_transfer</t>
+          <t>交河故城 -&gt; 罗布人村寨；charter_car</t>
         </is>
       </c>
     </row>
@@ -5688,7 +5688,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>罗布人村寨 -&gt; 库车王府；mixed_transfer</t>
+          <t>罗布人村寨 -&gt; 库车王府；rental_car</t>
         </is>
       </c>
     </row>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>罗布人村寨 -&gt; 库车王府；mixed_transfer</t>
+          <t>罗布人村寨 -&gt; 库车王府；rental_car</t>
         </is>
       </c>
     </row>
@@ -5878,7 +5878,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>库车王府 -&gt; 艾提尕尔清真寺；mixed_transfer</t>
+          <t>库车王府 -&gt; 艾提尕尔清真寺；charter_car</t>
         </is>
       </c>
     </row>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>库车王府 -&gt; 艾提尕尔清真寺；mixed_transfer</t>
+          <t>库车王府 -&gt; 艾提尕尔清真寺；charter_car</t>
         </is>
       </c>
     </row>
@@ -6134,7 +6134,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>艾提尕尔清真寺 -&gt; 喀什古城；mixed_transfer</t>
+          <t>艾提尕尔清真寺 -&gt; 喀什古城；taxi_transfer</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -6730,7 +6730,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -6920,7 +6920,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>北庭故城遗址 -&gt; 高昌故城；mixed_transfer</t>
+          <t>北庭故城遗址 -&gt; 高昌故城；rental_car</t>
         </is>
       </c>
     </row>
@@ -6982,7 +6982,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>北庭故城遗址 -&gt; 高昌故城；mixed_transfer</t>
+          <t>北庭故城遗址 -&gt; 高昌故城；rental_car</t>
         </is>
       </c>
     </row>
@@ -7176,7 +7176,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>高昌故城 -&gt; 克孜尔石窟；mixed_transfer</t>
+          <t>高昌故城 -&gt; 克孜尔石窟；charter_car</t>
         </is>
       </c>
     </row>
@@ -7238,7 +7238,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>高昌故城 -&gt; 克孜尔石窟；mixed_transfer</t>
+          <t>高昌故城 -&gt; 克孜尔石窟；charter_car</t>
         </is>
       </c>
     </row>
@@ -7300,7 +7300,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>高昌故城 -&gt; 克孜尔石窟；mixed_transfer</t>
+          <t>高昌故城 -&gt; 克孜尔石窟；charter_car</t>
         </is>
       </c>
     </row>
@@ -7494,7 +7494,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>克孜尔石窟 -&gt; 石头城遗址；mixed_transfer</t>
+          <t>克孜尔石窟 -&gt; 石头城遗址；charter_car</t>
         </is>
       </c>
     </row>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>克孜尔石窟 -&gt; 石头城遗址；mixed_transfer</t>
+          <t>克孜尔石窟 -&gt; 石头城遗址；charter_car</t>
         </is>
       </c>
     </row>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>石头城遗址 -&gt; 香妃园；mixed_transfer</t>
+          <t>石头城遗址 -&gt; 香妃园；rental_car</t>
         </is>
       </c>
     </row>
@@ -7944,7 +7944,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>石头城遗址 -&gt; 香妃园；mixed_transfer</t>
+          <t>石头城遗址 -&gt; 香妃园；rental_car</t>
         </is>
       </c>
     </row>
@@ -8242,7 +8242,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -8300,7 +8300,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -8358,7 +8358,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -8416,7 +8416,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>Q3-V2稳健主推预留5天项目缓冲</t>
+          <t>Q3-V2成本敏感均衡策略预留5天项目缓冲</t>
         </is>
       </c>
     </row>
@@ -13139,7 +13139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13188,6 +13188,11 @@
           <t>selection_status</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>strategy_tier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -13223,6 +13228,11 @@
           <t>normal_or_controlled_option</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>常规可控选项</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -13255,7 +13265,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>balanced_robust_main</t>
+          <t>cost_sensitive_balanced_strategy</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>成本敏感均衡策略</t>
         </is>
       </c>
     </row>
@@ -13290,7 +13305,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>cost_sensitive_extreme_backup</t>
+          <t>cost_sensitive_high_risk_backup</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>成本敏感高风险备选</t>
         </is>
       </c>
     </row>
@@ -13325,7 +13345,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>extreme_risk_backup</t>
+          <t>high_reliability_execution_strategy</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>高可靠执行策略</t>
         </is>
       </c>
     </row>
@@ -13360,7 +13385,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>compound_extreme_contingency</t>
+          <t>compound_extreme_contingency_plan</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>复合极端预案</t>
         </is>
       </c>
     </row>

</xml_diff>